<commit_message>
reorganizace slozek pred kopirovanim do EE
</commit_message>
<xml_diff>
--- a/data/input_denniData.xlsx
+++ b/data/input_denniData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krizova\Documents\R\02 cenoveKalkukacky\_vyvoj\shiny_app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42B6DEF-B2B4-47F7-83FB-A91FCC2050F3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB65501-B6C5-44A1-B9F3-C72C413F31A1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,9 +31,6 @@
     <t>low_spot</t>
   </si>
   <si>
-    <t>indikator</t>
-  </si>
-  <si>
     <t>hodnota</t>
   </si>
   <si>
@@ -53,6 +50,9 @@
   </si>
   <si>
     <t>marzeDop</t>
+  </si>
+  <si>
+    <t>parametr</t>
   </si>
 </sst>
 </file>
@@ -403,10 +403,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -419,7 +419,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2">
         <v>0.35</v>
@@ -427,7 +427,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="3">
         <f>B2+B3</f>
@@ -436,7 +436,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -444,7 +444,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2">
         <v>1.2</v>
@@ -452,7 +452,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2">
         <v>1.2</v>
@@ -460,7 +460,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2">
         <v>6</v>

</xml_diff>